<commit_message>
Align Phase 1 error registry and expected results
</commit_message>
<xml_diff>
--- a/hanbit_mvp_dataset_phase1/90_expected_results.xlsx
+++ b/hanbit_mvp_dataset_phase1/90_expected_results.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="validation_summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="validation_summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'validation_summary'!$A$1:$D$33</definedName>
@@ -924,7 +924,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1012,7 +1012,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">

</xml_diff>